<commit_message>
All results on alpha band
</commit_message>
<xml_diff>
--- a/results_coherence.xlsx
+++ b/results_coherence.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://epflch-my.sharepoint.com/personal/martina_baroffio_epfl_ch/Documents/EPFL/MA1/ML/ML4Science/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_74212A8AD049320F62355476585DCE3A874707F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D3344F0-687C-4C96-B917-91E0BCD7F7C8}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_573D3848504BB40E62355476585DCE3A874663F4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A0E43B0-77A5-4493-8261-D5B996CA0258}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="82">
   <si>
     <t>Model</t>
   </si>
@@ -164,6 +164,108 @@
   </si>
   <si>
     <t>0.1301</t>
+  </si>
+  <si>
+    <t>XGBoost</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 1.0, 'xgb__learning_rate': 0.05, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 500, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.8, 'xgb__learning_rate': 0.01, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.6, 'xgb__learning_rate': 0.1, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.8, 'xgb__learning_rate': 0.01, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 300, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.8, 'xgb__learning_rate': 0.05, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 300, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.6, 'xgb__learning_rate': 0.01, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 1.0}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 1.0, 'xgb__learning_rate': 0.01, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 1.0}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.6, 'xgb__learning_rate': 0.05, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.6, 'xgb__learning_rate': 0.01, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.6, 'xgb__learning_rate': 0.05, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 300, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 1.0, 'xgb__learning_rate': 0.1, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 300, 'xgb__subsample': 0.8}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.8, 'xgb__learning_rate': 0.01, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 500, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 1.0, 'xgb__learning_rate': 0.05, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 1.0, 'xgb__learning_rate': 0.1, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 0.8}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.6, 'xgb__learning_rate': 0.01, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 500, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.8, 'xgb__learning_rate': 0.1, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 500, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.6, 'xgb__learning_rate': 0.1, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 0.8}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.6, 'xgb__learning_rate': 0.01, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 300, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.8, 'xgb__learning_rate': 0.1, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.6, 'xgb__learning_rate': 0.1, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 500, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 1.0, 'xgb__learning_rate': 0.05, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 300, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.6, 'xgb__learning_rate': 0.01, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 0.8}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.8, 'xgb__learning_rate': 0.01, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 1.0}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.6, 'xgb__learning_rate': 0.01, 'xgb__max_depth': 3, 'xgb__min_child_weight': 5, 'xgb__n_estimators': 100, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 1.0, 'xgb__learning_rate': 0.05, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 0.8}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.8, 'xgb__learning_rate': 0.05, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.6, 'xgb__learning_rate': 0.1, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 300, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.8, 'xgb__learning_rate': 0.05, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 0.8}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 1.0, 'xgb__learning_rate': 0.01, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 500, 'xgb__subsample': 0.8}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.6, 'xgb__learning_rate': 0.05, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 500, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 1.0, 'xgb__learning_rate': 0.1, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>0.5312</t>
+  </si>
+  <si>
+    <t>0.1309</t>
   </si>
 </sst>
 </file>
@@ -526,7 +628,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F151"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -1967,6 +2069,712 @@
         <v>47</v>
       </c>
     </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>48</v>
+      </c>
+      <c r="B102" t="s">
+        <v>49</v>
+      </c>
+      <c r="C102">
+        <v>0.72579365079365077</v>
+      </c>
+      <c r="D102">
+        <v>0.48484848484848492</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>48</v>
+      </c>
+      <c r="B103" t="s">
+        <v>50</v>
+      </c>
+      <c r="C103">
+        <v>0.65357142857142858</v>
+      </c>
+      <c r="D103">
+        <v>0.51515151515151514</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>48</v>
+      </c>
+      <c r="B104" t="s">
+        <v>51</v>
+      </c>
+      <c r="C104">
+        <v>0.60277777777777775</v>
+      </c>
+      <c r="D104">
+        <v>0.56060606060606055</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>48</v>
+      </c>
+      <c r="B105" t="s">
+        <v>52</v>
+      </c>
+      <c r="C105">
+        <v>0.59603174603174602</v>
+      </c>
+      <c r="D105">
+        <v>0.60606060606060597</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
+        <v>48</v>
+      </c>
+      <c r="B106" t="s">
+        <v>53</v>
+      </c>
+      <c r="C106">
+        <v>0.64682539682539675</v>
+      </c>
+      <c r="D106">
+        <v>0.5757575757575758</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>48</v>
+      </c>
+      <c r="B107" t="s">
+        <v>54</v>
+      </c>
+      <c r="C107">
+        <v>0.69761904761904769</v>
+      </c>
+      <c r="D107">
+        <v>0.53030303030303028</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
+        <v>48</v>
+      </c>
+      <c r="B108" t="s">
+        <v>55</v>
+      </c>
+      <c r="C108">
+        <v>0.60793650793650789</v>
+      </c>
+      <c r="D108">
+        <v>0.69696969696969702</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
+        <v>48</v>
+      </c>
+      <c r="B109" t="s">
+        <v>56</v>
+      </c>
+      <c r="C109">
+        <v>0.6968253968253969</v>
+      </c>
+      <c r="D109">
+        <v>0.69696969696969702</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
+        <v>48</v>
+      </c>
+      <c r="B110" t="s">
+        <v>56</v>
+      </c>
+      <c r="C110">
+        <v>0.6515873015873016</v>
+      </c>
+      <c r="D110">
+        <v>0.53030303030303028</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
+        <v>48</v>
+      </c>
+      <c r="B111" t="s">
+        <v>57</v>
+      </c>
+      <c r="C111">
+        <v>0.70119047619047625</v>
+      </c>
+      <c r="D111">
+        <v>0.59090909090909094</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
+        <v>48</v>
+      </c>
+      <c r="B112" t="s">
+        <v>54</v>
+      </c>
+      <c r="C112">
+        <v>0.60476190476190483</v>
+      </c>
+      <c r="D112">
+        <v>0.43939393939393928</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
+        <v>48</v>
+      </c>
+      <c r="B113" t="s">
+        <v>58</v>
+      </c>
+      <c r="C113">
+        <v>0.64047619047619053</v>
+      </c>
+      <c r="D113">
+        <v>0.69696969696969702</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
+        <v>48</v>
+      </c>
+      <c r="B114" t="s">
+        <v>59</v>
+      </c>
+      <c r="C114">
+        <v>0.58611111111111114</v>
+      </c>
+      <c r="D114">
+        <v>0.48484848484848492</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
+        <v>48</v>
+      </c>
+      <c r="B115" t="s">
+        <v>51</v>
+      </c>
+      <c r="C115">
+        <v>0.74365079365079367</v>
+      </c>
+      <c r="D115">
+        <v>0.5757575757575758</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
+        <v>48</v>
+      </c>
+      <c r="B116" t="s">
+        <v>60</v>
+      </c>
+      <c r="C116">
+        <v>0.67738095238095231</v>
+      </c>
+      <c r="D116">
+        <v>0.43939393939393928</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
+        <v>48</v>
+      </c>
+      <c r="B117" t="s">
+        <v>61</v>
+      </c>
+      <c r="C117">
+        <v>0.59246031746031746</v>
+      </c>
+      <c r="D117">
+        <v>0.31818181818181818</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
+        <v>48</v>
+      </c>
+      <c r="B118" t="s">
+        <v>56</v>
+      </c>
+      <c r="C118">
+        <v>0.65952380952380951</v>
+      </c>
+      <c r="D118">
+        <v>0.31818181818181818</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
+        <v>48</v>
+      </c>
+      <c r="B119" t="s">
+        <v>62</v>
+      </c>
+      <c r="C119">
+        <v>0.67896825396825411</v>
+      </c>
+      <c r="D119">
+        <v>0.65151515151515149</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A120" t="s">
+        <v>48</v>
+      </c>
+      <c r="B120" t="s">
+        <v>63</v>
+      </c>
+      <c r="C120">
+        <v>0.55634920634920637</v>
+      </c>
+      <c r="D120">
+        <v>0.69696969696969702</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A121" t="s">
+        <v>48</v>
+      </c>
+      <c r="B121" t="s">
+        <v>64</v>
+      </c>
+      <c r="C121">
+        <v>0.68492063492063482</v>
+      </c>
+      <c r="D121">
+        <v>0.43939393939393928</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A122" t="s">
+        <v>48</v>
+      </c>
+      <c r="B122" t="s">
+        <v>65</v>
+      </c>
+      <c r="C122">
+        <v>0.53174603174603174</v>
+      </c>
+      <c r="D122">
+        <v>0.62121212121212122</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A123" t="s">
+        <v>48</v>
+      </c>
+      <c r="B123" t="s">
+        <v>66</v>
+      </c>
+      <c r="C123">
+        <v>0.57658730158730165</v>
+      </c>
+      <c r="D123">
+        <v>0.60606060606060597</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A124" t="s">
+        <v>48</v>
+      </c>
+      <c r="B124" t="s">
+        <v>67</v>
+      </c>
+      <c r="C124">
+        <v>0.76071428571428579</v>
+      </c>
+      <c r="D124">
+        <v>0.22727272727272729</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A125" t="s">
+        <v>48</v>
+      </c>
+      <c r="B125" t="s">
+        <v>56</v>
+      </c>
+      <c r="C125">
+        <v>0.77579365079365081</v>
+      </c>
+      <c r="D125">
+        <v>0.45454545454545447</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A126" t="s">
+        <v>48</v>
+      </c>
+      <c r="B126" t="s">
+        <v>68</v>
+      </c>
+      <c r="C126">
+        <v>0.62341269841269842</v>
+      </c>
+      <c r="D126">
+        <v>0.60606060606060597</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A127" t="s">
+        <v>48</v>
+      </c>
+      <c r="B127" t="s">
+        <v>69</v>
+      </c>
+      <c r="C127">
+        <v>0.71349206349206351</v>
+      </c>
+      <c r="D127">
+        <v>0.45454545454545447</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A128" t="s">
+        <v>48</v>
+      </c>
+      <c r="B128" t="s">
+        <v>70</v>
+      </c>
+      <c r="C128">
+        <v>0.71031746031746035</v>
+      </c>
+      <c r="D128">
+        <v>0.78787878787878785</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A129" t="s">
+        <v>48</v>
+      </c>
+      <c r="B129" t="s">
+        <v>51</v>
+      </c>
+      <c r="C129">
+        <v>0.65595238095238095</v>
+      </c>
+      <c r="D129">
+        <v>0.65151515151515149</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A130" t="s">
+        <v>48</v>
+      </c>
+      <c r="B130" t="s">
+        <v>71</v>
+      </c>
+      <c r="C130">
+        <v>0.74285714285714288</v>
+      </c>
+      <c r="D130">
+        <v>0.5757575757575758</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A131" t="s">
+        <v>48</v>
+      </c>
+      <c r="B131" t="s">
+        <v>72</v>
+      </c>
+      <c r="C131">
+        <v>0.5</v>
+      </c>
+      <c r="D131">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A132" t="s">
+        <v>48</v>
+      </c>
+      <c r="B132" t="s">
+        <v>51</v>
+      </c>
+      <c r="C132">
+        <v>0.63293650793650791</v>
+      </c>
+      <c r="D132">
+        <v>0.2121212121212121</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A133" t="s">
+        <v>48</v>
+      </c>
+      <c r="B133" t="s">
+        <v>73</v>
+      </c>
+      <c r="C133">
+        <v>0.69761904761904747</v>
+      </c>
+      <c r="D133">
+        <v>0.48484848484848492</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A134" t="s">
+        <v>48</v>
+      </c>
+      <c r="B134" t="s">
+        <v>50</v>
+      </c>
+      <c r="C134">
+        <v>0.69603174603174611</v>
+      </c>
+      <c r="D134">
+        <v>0.53030303030303028</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A135" t="s">
+        <v>48</v>
+      </c>
+      <c r="B135" t="s">
+        <v>74</v>
+      </c>
+      <c r="C135">
+        <v>0.78769841269841268</v>
+      </c>
+      <c r="D135">
+        <v>0.53030303030303028</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A136" t="s">
+        <v>48</v>
+      </c>
+      <c r="B136" t="s">
+        <v>75</v>
+      </c>
+      <c r="C136">
+        <v>0.67619047619047612</v>
+      </c>
+      <c r="D136">
+        <v>0.43939393939393928</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A137" t="s">
+        <v>48</v>
+      </c>
+      <c r="B137" t="s">
+        <v>73</v>
+      </c>
+      <c r="C137">
+        <v>0.625</v>
+      </c>
+      <c r="D137">
+        <v>0.74242424242424243</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A138" t="s">
+        <v>48</v>
+      </c>
+      <c r="B138" t="s">
+        <v>58</v>
+      </c>
+      <c r="C138">
+        <v>0.74642857142857144</v>
+      </c>
+      <c r="D138">
+        <v>0.78787878787878785</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A139" t="s">
+        <v>48</v>
+      </c>
+      <c r="B139" t="s">
+        <v>76</v>
+      </c>
+      <c r="C139">
+        <v>0.72817460317460325</v>
+      </c>
+      <c r="D139">
+        <v>0.39393939393939392</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A140" t="s">
+        <v>48</v>
+      </c>
+      <c r="B140" t="s">
+        <v>50</v>
+      </c>
+      <c r="C140">
+        <v>0.70039682539682546</v>
+      </c>
+      <c r="D140">
+        <v>0.60606060606060597</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A141" t="s">
+        <v>48</v>
+      </c>
+      <c r="B141" t="s">
+        <v>77</v>
+      </c>
+      <c r="C141">
+        <v>0.62182539682539684</v>
+      </c>
+      <c r="D141">
+        <v>0.43939393939393928</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A142" t="s">
+        <v>48</v>
+      </c>
+      <c r="B142" t="s">
+        <v>62</v>
+      </c>
+      <c r="C142">
+        <v>0.6968253968253969</v>
+      </c>
+      <c r="D142">
+        <v>0.62121212121212122</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A143" t="s">
+        <v>48</v>
+      </c>
+      <c r="B143" t="s">
+        <v>50</v>
+      </c>
+      <c r="C143">
+        <v>0.86190476190476184</v>
+      </c>
+      <c r="D143">
+        <v>0.27272727272727271</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A144" t="s">
+        <v>48</v>
+      </c>
+      <c r="B144" t="s">
+        <v>57</v>
+      </c>
+      <c r="C144">
+        <v>0.66785714285714282</v>
+      </c>
+      <c r="D144">
+        <v>0.56060606060606055</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A145" t="s">
+        <v>48</v>
+      </c>
+      <c r="B145" t="s">
+        <v>78</v>
+      </c>
+      <c r="C145">
+        <v>0.71547619047619049</v>
+      </c>
+      <c r="D145">
+        <v>0.48484848484848492</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A146" t="s">
+        <v>48</v>
+      </c>
+      <c r="B146" t="s">
+        <v>77</v>
+      </c>
+      <c r="C146">
+        <v>0.72658730158730156</v>
+      </c>
+      <c r="D146">
+        <v>0.53030303030303028</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A147" t="s">
+        <v>48</v>
+      </c>
+      <c r="B147" t="s">
+        <v>51</v>
+      </c>
+      <c r="C147">
+        <v>0.55436507936507951</v>
+      </c>
+      <c r="D147">
+        <v>0.65151515151515149</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A148" t="s">
+        <v>48</v>
+      </c>
+      <c r="B148" t="s">
+        <v>79</v>
+      </c>
+      <c r="C148">
+        <v>0.794047619047619</v>
+      </c>
+      <c r="D148">
+        <v>0.45454545454545447</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A149" t="s">
+        <v>48</v>
+      </c>
+      <c r="B149" t="s">
+        <v>61</v>
+      </c>
+      <c r="C149">
+        <v>0.68690476190476202</v>
+      </c>
+      <c r="D149">
+        <v>0.53030303030303028</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
+        <v>48</v>
+      </c>
+      <c r="B150" t="s">
+        <v>63</v>
+      </c>
+      <c r="C150">
+        <v>0.65079365079365081</v>
+      </c>
+      <c r="D150">
+        <v>0.56060606060606055</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A151" t="s">
+        <v>48</v>
+      </c>
+      <c r="B151" t="s">
+        <v>54</v>
+      </c>
+      <c r="C151">
+        <v>0.66865079365079361</v>
+      </c>
+      <c r="D151">
+        <v>0.39393939393939392</v>
+      </c>
+      <c r="E151" t="s">
+        <v>80</v>
+      </c>
+      <c r="F151" t="s">
+        <v>81</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>